<commit_message>
Updated Excel output if weight charges are zero
</commit_message>
<xml_diff>
--- a/public/finance/Shipment Charges View.xlsx
+++ b/public/finance/Shipment Charges View.xlsx
@@ -74,10 +74,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
@@ -88,10 +85,10 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+      <alignment vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="1" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+      <alignment vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -438,22 +435,16 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="1">
-        <v>22322846347147</v>
+        <v>202202368447</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>40000</v>
       </c>
       <c r="C2">
-        <v>1800</v>
-      </c>
-      <c r="D2">
-        <v>160.0</v>
+        <v>5000</v>
       </c>
       <c r="E2">
-        <v>0.0</v>
-      </c>
-      <c r="H2">
-        <v>57.6</v>
+        <v>100.0</v>
       </c>
     </row>
   </sheetData>
@@ -469,5 +460,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>